<commit_message>
Added missing redirect to Excel file
</commit_message>
<xml_diff>
--- a/website/home/migrations/0116_create_redirects_for_broken_pdf_links.xlsx
+++ b/website/home/migrations/0116_create_redirects_for_broken_pdf_links.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30105"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BACBD6E-8D34-4323-9A0E-7A2C1F5D2268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AB708EA-E7D4-43C6-99D6-62FF871865B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>From</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>/files/documents/Administrative_Order_2022-01_Repealed.pdf</t>
+  </si>
+  <si>
+    <t>/resources/administrative_orders/Administrative_Order_2022-01.pdf</t>
   </si>
   <si>
     <t>/rules/Title_II.pdf</t>
@@ -171,10 +174,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -489,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="63.42578125" customWidth="1"/>
@@ -512,10 +514,10 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2" t="s">
@@ -523,10 +525,10 @@
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
@@ -534,10 +536,10 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
       <c r="C4" t="s">
@@ -545,10 +547,10 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="2" t="s">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>12</v>
       </c>
       <c r="C5" t="s">
@@ -556,10 +558,10 @@
       </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6" t="s">
@@ -567,10 +569,10 @@
       </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
+      <c r="A7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="C7" t="s">
@@ -578,10 +580,10 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>18</v>
       </c>
       <c r="C8" t="s">
@@ -589,10 +591,10 @@
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>20</v>
       </c>
       <c r="C9" t="s">
@@ -600,10 +602,10 @@
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>22</v>
       </c>
       <c r="C10" t="s">
@@ -611,10 +613,10 @@
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="2" t="s">
+      <c r="A11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>24</v>
       </c>
       <c r="C11" t="s">
@@ -622,46 +624,57 @@
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="2" t="s">
+      <c r="B13" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
         <v>28</v>
       </c>
-      <c r="C13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="2" t="s">
+      <c r="B14" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="2" t="s">
+      <c r="B15" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
         <v>32</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed redirect for /resources/administrative_orders/Administrative_Order_2022-01.pdf
</commit_message>
<xml_diff>
--- a/website/home/migrations/0116_create_redirects_for_broken_pdf_links.xlsx
+++ b/website/home/migrations/0116_create_redirects_for_broken_pdf_links.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30105"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1AB708EA-E7D4-43C6-99D6-62FF871865B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2922B67F-AB40-43E2-8D16-98B0E0CF6127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
   <si>
     <t>From</t>
   </si>
@@ -105,10 +105,13 @@
     <t>/resources/administrative_orders/Administrative_Order_2021-02.pdf</t>
   </si>
   <si>
+    <t>/files/documents/Administrative_Order_2021-02_REPEALED.pdf</t>
+  </si>
+  <si>
+    <t>/resources/administrative_orders/Administrative_Order_2022-01.pdf</t>
+  </si>
+  <si>
     <t>/files/documents/Administrative_Order_2022-01_Repealed.pdf</t>
-  </si>
-  <si>
-    <t>/resources/administrative_orders/Administrative_Order_2022-01.pdf</t>
   </si>
   <si>
     <t>/rules/Title_II.pdf</t>
@@ -174,9 +177,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,7 +620,7 @@
       <c r="A11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C11" t="s">
@@ -628,7 +632,7 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
@@ -636,10 +640,10 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
         <v>6</v>
@@ -647,10 +651,10 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
         <v>6</v>
@@ -658,10 +662,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
@@ -669,10 +673,10 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>

</xml_diff>